<commit_message>
Update kaspa_buys.xlsx after running on 2026-03-06
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -898,6 +898,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>03/06/2026</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1606.672999999995</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.03080900718441161</v>
+      </c>
+      <c r="D30" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-03-13
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -914,6 +914,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>03/13/2026</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1603.520000000004</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.03086958690880056</v>
+      </c>
+      <c r="D31" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-03-20
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -930,6 +930,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>03/20/2026</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1301.290000000001</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0.03803917650946366</v>
+      </c>
+      <c r="D32" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-03-27
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -946,6 +946,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>03/27/2026</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1361.277999999998</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0.03636288840339744</v>
+      </c>
+      <c r="D33" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-04-03
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -962,6 +962,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>04/03/2026</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1561.133999999998</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0.03170772015727033</v>
+      </c>
+      <c r="D34" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-04-10
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -978,6 +978,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>04/10/2026</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1519.988000000005</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0.03256604657405179</v>
+      </c>
+      <c r="D35" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-04-17
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -994,6 +994,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>04/17/2026</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1446.805999999997</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0.0342132946642467</v>
+      </c>
+      <c r="D36" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-04-24
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1010,6 +1010,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>04/24/2026</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1432.065999999999</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0.0345654460059802</v>
+      </c>
+      <c r="D37" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-05-01
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1026,6 +1026,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>05/01/2026</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1508.760000000002</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0.03280839895013119</v>
+      </c>
+      <c r="D38" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-05-08
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1042,6 +1042,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>05/08/2026</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1391.417000000001</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0.03557524451692048</v>
+      </c>
+      <c r="D39" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-05-15
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1058,6 +1058,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>05/15/2026</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1294.417999999998</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0.03824112458263102</v>
+      </c>
+      <c r="D40" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-05-22
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1074,6 +1074,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>05/22/2026</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1391.811999999998</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0.03556514816656278</v>
+      </c>
+      <c r="D41" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-05-29
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1090,6 +1090,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>05/29/2026</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1584.344000000005</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0.03124321485737937</v>
+      </c>
+      <c r="D42" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-06-05
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1106,6 +1106,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>06/05/2026</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1658.869999999995</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0.02983958960014958</v>
+      </c>
+      <c r="D43" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-06-12
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1122,6 +1122,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>06/12/2026</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1578.731</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0.0313542965837752</v>
+      </c>
+      <c r="D44" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-06-19
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D44"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1138,6 +1138,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>06/19/2026</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1611.427000000003</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0.03071811506199158</v>
+      </c>
+      <c r="D45" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-06-26
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1154,6 +1154,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>06/26/2026</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1775.980000000003</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0.02787193549476904</v>
+      </c>
+      <c r="D46" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-07-03
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1170,6 +1170,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1591.98401</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0.03109327712405855</v>
+      </c>
+      <c r="D47" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-07-10
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1186,6 +1186,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1655.508999999998</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0.0299001696759124</v>
+      </c>
+      <c r="D48" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-07-17
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1202,6 +1202,22 @@
         <v>50</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>07/17/2026</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>867.2969999999987</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0.02853693717377097</v>
+      </c>
+      <c r="D49" t="n">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-07-24
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1218,6 +1218,22 @@
         <v>25</v>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>07/24/2026</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>875.3500000000058</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0.02827440452390454</v>
+      </c>
+      <c r="D50" t="n">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-07-31
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1234,6 +1234,22 @@
         <v>25</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>07/31/2026</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>887.3930000000037</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0.02789068653910939</v>
+      </c>
+      <c r="D51" t="n">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-08-07
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1250,6 +1250,22 @@
         <v>25</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>955.9209999999948</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0.02589126088871375</v>
+      </c>
+      <c r="D52" t="n">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-08-14
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:D53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1266,6 +1266,22 @@
         <v>25</v>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>08/14/2026</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>969.1500000000015</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0.02553784243925085</v>
+      </c>
+      <c r="D53" t="n">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-08-21
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D53"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1282,6 +1282,22 @@
         <v>25</v>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>08/21/2026</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>872.2350000000006</v>
+      </c>
+      <c r="C54" t="n">
+        <v>0.02837538048805652</v>
+      </c>
+      <c r="D54" t="n">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-08-28
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D54"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1298,6 +1298,22 @@
         <v>25</v>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>08/28/2026</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>838.5149999999994</v>
+      </c>
+      <c r="C55" t="n">
+        <v>0.02951646661061522</v>
+      </c>
+      <c r="D55" t="n">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-09-04
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1314,6 +1314,22 @@
         <v>25</v>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>827.474000000002</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0.02991030533889879</v>
+      </c>
+      <c r="D56" t="n">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update kaspa_buys.xlsx after running on 2026-09-11
</commit_message>
<xml_diff>
--- a/data/kaspa_buys.xlsx
+++ b/data/kaspa_buys.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D56"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1330,6 +1330,22 @@
         <v>25</v>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>09/11/2026</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>690.8059999999969</v>
+      </c>
+      <c r="C57" t="n">
+        <v>0.03582771429315917</v>
+      </c>
+      <c r="D57" t="n">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>